<commit_message>
updated to use mse5, goal set to black river at pocahontas, and just 100yr freq run
</commit_message>
<xml_diff>
--- a/presentation/HMR DAD curves.xlsx
+++ b/presentation/HMR DAD curves.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\py\freq_flow_isohyet_optimizer\presentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5283602D-EBC3-4576-BC71-E19F764F7530}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE015EAF-E853-4E36-A8FD-3C9FF386B48D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{FA2728A9-FF84-4620-AD07-5750A2971436}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{FA2728A9-FF84-4620-AD07-5750A2971436}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="32">
   <si>
     <t>Area</t>
   </si>
@@ -119,6 +118,24 @@
   </si>
   <si>
     <t>Current River Internal</t>
+  </si>
+  <si>
+    <t>Current River Internal-B</t>
+  </si>
+  <si>
+    <t>Murray Creek-Black Riv InB</t>
+  </si>
+  <si>
+    <t>Fourche River-B</t>
+  </si>
+  <si>
+    <t>Fourche River</t>
+  </si>
+  <si>
+    <t>Big Running Water Creek-Bla</t>
+  </si>
+  <si>
+    <t>Outlet Spring River Internal</t>
   </si>
 </sst>
 </file>
@@ -162,12 +179,24 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -197,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -221,6 +250,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2390,93 +2422,181 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5142C2C-ACEF-4DFE-A7FB-DF5DE87B7F9A}">
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.42578125" customWidth="1"/>
+    <col min="3" max="3" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+    </row>
+    <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" s="10"/>
+    </row>
+    <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="C12" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="C13" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>25</v>
+        <v>14</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C17" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="3:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="3:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C20" s="11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="3:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C21" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="22" spans="3:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="9" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C1:C22">
+    <sortCondition ref="C1:C22"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>